<commit_message>
feat: display partially eligible status, FOIR cap, and red caution breach remarks on customer offer letter and shareable PDF
</commit_message>
<xml_diff>
--- a/Quickfinsure_Bank_Policy_Cards.xlsx
+++ b/Quickfinsure_Bank_Policy_Cards.xlsx
@@ -8,15 +8,18 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/120435612014f931/Tài liệu/Important Sheet/Anitigravity Projects/Quickfinsure/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3" documentId="11_3F12451216A80BE399152093C815A669B06F13AD" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{47ADCCC5-9E99-47AD-887D-B7B1C3475FAD}"/>
+  <xr:revisionPtr revIDLastSave="5" documentId="11_3F12451216A80BE399152093C815A669B06F13AD" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E0F8A543-6637-4812-A91B-28125BE3C45B}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Bank Policies Summary" sheetId="1" r:id="rId1"/>
     <sheet name="Eligibility &amp; Dynamic Rules" sheetId="2" r:id="rId2"/>
     <sheet name="CIBIL Rate Matrix" sheetId="3" r:id="rId3"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'CIBIL Rate Matrix'!$A$1:$K$20</definedName>
+  </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
@@ -1702,6 +1705,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:K20"/>
   <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -1858,7 +1862,7 @@
         <v>100000000</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>33</v>
       </c>
@@ -1893,7 +1897,7 @@
         <v>150000000</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>33</v>
       </c>
@@ -1928,7 +1932,7 @@
         <v>150000000</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>33</v>
       </c>
@@ -1963,7 +1967,7 @@
         <v>150000000</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>37</v>
       </c>
@@ -1998,7 +2002,7 @@
         <v>4000000</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>37</v>
       </c>
@@ -2033,7 +2037,7 @@
         <v>4000000</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>37</v>
       </c>
@@ -2068,7 +2072,7 @@
         <v>4000000</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>44</v>
       </c>
@@ -2103,7 +2107,7 @@
         <v>3500000</v>
       </c>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>44</v>
       </c>
@@ -2138,7 +2142,7 @@
         <v>3500000</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>49</v>
       </c>
@@ -2173,7 +2177,7 @@
         <v>150000000</v>
       </c>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>49</v>
       </c>
@@ -2208,7 +2212,7 @@
         <v>150000000</v>
       </c>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>49</v>
       </c>
@@ -2243,7 +2247,7 @@
         <v>150000000</v>
       </c>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>53</v>
       </c>
@@ -2278,7 +2282,7 @@
         <v>7500000</v>
       </c>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>53</v>
       </c>
@@ -2313,7 +2317,7 @@
         <v>7500000</v>
       </c>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>60</v>
       </c>
@@ -2348,7 +2352,7 @@
         <v>50000000</v>
       </c>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>60</v>
       </c>
@@ -2383,7 +2387,7 @@
         <v>50000000</v>
       </c>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>60</v>
       </c>
@@ -2419,6 +2423,13 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:K20" xr:uid="{00000000-0001-0000-0200-000000000000}">
+    <filterColumn colId="0">
+      <filters>
+        <filter val="HDFC Bank"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
     <ignoredError sqref="A1:K20" numberStoredAsText="1"/>

</xml_diff>